<commit_message>
Add Dr. Amteshwar Singh lecture and fix Vimeo upload dedup
- Append Dr. Amteshwar Singh's Oct 2026 lecture week to consultant_vimeo.csv,
  download from Zoom, upload to Vimeo, and add the links to vimeo_links.xlsx
  / vimeo_links_omit.xlsx.
- vimeo_upload.py: use consultant_vimeo.csv's own "Vimeo URI"/"Vimeoリンク"
  columns as the primary dedup check instead of matching titles against
  Vimeo's live catalog, which was unreliable (128-char title truncation on
  upload, and duplicate-titled videos colliding in the lookup dict) and had
  caused repeated duplicate uploads. Results are now written back into the
  source CSV automatically after each run.
- Backfill the new columns for all existing rows and clean up the 40
  historical duplicate videos this bug had created on Vimeo.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/vimeo_links.xlsx
+++ b/vimeo_links.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Vimeo Links" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vimeo Links" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -64,7 +64,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -85,6 +85,18 @@
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
   </cellXfs>
@@ -452,7 +464,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F115"/>
+  <dimension ref="A1:F148"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -551,7 +563,7 @@
       </c>
       <c r="F3" s="6" t="inlineStr">
         <is>
-          <t>https://vimeo.com/1154202805</t>
+          <t>https://vimeo.com/1154200765</t>
         </is>
       </c>
     </row>
@@ -583,7 +595,7 @@
       </c>
       <c r="F4" s="7" t="inlineStr">
         <is>
-          <t>https://vimeo.com/1154202922</t>
+          <t>https://vimeo.com/1154200948</t>
         </is>
       </c>
     </row>
@@ -647,7 +659,7 @@
       </c>
       <c r="F6" s="7" t="inlineStr">
         <is>
-          <t>https://vimeo.com/1154203273</t>
+          <t>https://vimeo.com/1154203167</t>
         </is>
       </c>
     </row>
@@ -675,7 +687,7 @@
       <c r="E7" s="4" t="inlineStr"/>
       <c r="F7" s="6" t="inlineStr">
         <is>
-          <t>https://vimeo.com/1154203273</t>
+          <t>https://vimeo.com/1154203167</t>
         </is>
       </c>
     </row>
@@ -2859,7 +2871,7 @@
       </c>
       <c r="F80" s="7" t="inlineStr">
         <is>
-          <t>https://vimeo.com/1192449734</t>
+          <t>https://vimeo.com/1177162061</t>
         </is>
       </c>
     </row>
@@ -2891,7 +2903,7 @@
       </c>
       <c r="F81" s="6" t="inlineStr">
         <is>
-          <t>https://vimeo.com/1192449909</t>
+          <t>https://vimeo.com/1177162237</t>
         </is>
       </c>
     </row>
@@ -2923,7 +2935,7 @@
       </c>
       <c r="F82" s="7" t="inlineStr">
         <is>
-          <t>https://vimeo.com/1192450070</t>
+          <t>https://vimeo.com/1177162517</t>
         </is>
       </c>
     </row>
@@ -2955,7 +2967,7 @@
       </c>
       <c r="F83" s="6" t="inlineStr">
         <is>
-          <t>https://vimeo.com/1192450190</t>
+          <t>https://vimeo.com/1177162727</t>
         </is>
       </c>
     </row>
@@ -3928,7 +3940,8 @@
       </c>
       <c r="C115" s="5" t="inlineStr">
         <is>
-          <t>Associate Professor Pediatric General and Thoracic Surgery, SSM Health Cardinal Glennon Children's Hospital St.Louis University School of Medicine</t>
+          <t>Associate Professor  Department of Internal Medicine
+         Division of Nephrology, St Louis University School of Medicine</t>
         </is>
       </c>
       <c r="D115" s="5" t="inlineStr">
@@ -3944,6 +3957,1046 @@
       <c r="F115" s="6" t="inlineStr">
         <is>
           <t>https://vimeo.com/1204027423</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="2" t="inlineStr">
+        <is>
+          <t>Kazuhito Hirata</t>
+        </is>
+      </c>
+      <c r="B116" s="2" t="inlineStr">
+        <is>
+          <t>循環器内科</t>
+        </is>
+      </c>
+      <c r="C116" s="3" t="inlineStr">
+        <is>
+          <t>社会福祉法人友愛会 友愛医療センター</t>
+        </is>
+      </c>
+      <c r="D116" s="3" t="inlineStr">
+        <is>
+          <t>JVP (Jugular Venous Pressure and Apex Beat)</t>
+        </is>
+      </c>
+      <c r="E116" s="2" t="inlineStr">
+        <is>
+          <t>353300</t>
+        </is>
+      </c>
+      <c r="F116" s="7" t="inlineStr">
+        <is>
+          <t>https://vimeo.com/1214920052</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="4" t="inlineStr">
+        <is>
+          <t>Kazuhito Hirata</t>
+        </is>
+      </c>
+      <c r="B117" s="4" t="inlineStr">
+        <is>
+          <t>循環器内科</t>
+        </is>
+      </c>
+      <c r="C117" s="5" t="inlineStr">
+        <is>
+          <t>社会福祉法人友愛会 友愛医療センター</t>
+        </is>
+      </c>
+      <c r="D117" s="5" t="inlineStr">
+        <is>
+          <t>Auscultation Workshop (Systolic Murmurs)</t>
+        </is>
+      </c>
+      <c r="E117" s="4" t="inlineStr">
+        <is>
+          <t>687971</t>
+        </is>
+      </c>
+      <c r="F117" s="6" t="inlineStr">
+        <is>
+          <t>https://vimeo.com/1214919031</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="2" t="inlineStr">
+        <is>
+          <t>Kazuhito Hirata</t>
+        </is>
+      </c>
+      <c r="B118" s="2" t="inlineStr">
+        <is>
+          <t>循環器内科</t>
+        </is>
+      </c>
+      <c r="C118" s="3" t="inlineStr">
+        <is>
+          <t>社会福祉法人友愛会 友愛医療センター</t>
+        </is>
+      </c>
+      <c r="D118" s="3" t="inlineStr">
+        <is>
+          <t>Physical examination workshop (Harvey)</t>
+        </is>
+      </c>
+      <c r="E118" s="2" t="inlineStr"/>
+      <c r="F118" s="2" t="inlineStr"/>
+    </row>
+    <row r="119">
+      <c r="A119" s="4" t="inlineStr">
+        <is>
+          <t>Kazuhito Hirata</t>
+        </is>
+      </c>
+      <c r="B119" s="4" t="inlineStr">
+        <is>
+          <t>循環器内科</t>
+        </is>
+      </c>
+      <c r="C119" s="5" t="inlineStr">
+        <is>
+          <t>社会福祉法人友愛会 友愛医療センター</t>
+        </is>
+      </c>
+      <c r="D119" s="5" t="inlineStr">
+        <is>
+          <t>Cardiac Auscultation (S2 and Extra Heart Sounds)</t>
+        </is>
+      </c>
+      <c r="E119" s="4" t="inlineStr">
+        <is>
+          <t>353300</t>
+        </is>
+      </c>
+      <c r="F119" s="6" t="inlineStr">
+        <is>
+          <t>https://vimeo.com/1214919113</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="2" t="inlineStr">
+        <is>
+          <t>Kazuhito Hirata</t>
+        </is>
+      </c>
+      <c r="B120" s="2" t="inlineStr">
+        <is>
+          <t>循環器内科</t>
+        </is>
+      </c>
+      <c r="C120" s="3" t="inlineStr">
+        <is>
+          <t>社会福祉法人友愛会 友愛医療センター</t>
+        </is>
+      </c>
+      <c r="D120" s="3" t="inlineStr">
+        <is>
+          <t>Auscultation Workshop (Extra Heart Sounds and S2)</t>
+        </is>
+      </c>
+      <c r="E120" s="2" t="inlineStr">
+        <is>
+          <t>687971</t>
+        </is>
+      </c>
+      <c r="F120" s="7" t="inlineStr">
+        <is>
+          <t>https://vimeo.com/1214919179</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="4" t="inlineStr">
+        <is>
+          <t>Kazuhito Hirata</t>
+        </is>
+      </c>
+      <c r="B121" s="4" t="inlineStr">
+        <is>
+          <t>循環器内科</t>
+        </is>
+      </c>
+      <c r="C121" s="5" t="inlineStr">
+        <is>
+          <t>社会福祉法人友愛会 友愛医療センター</t>
+        </is>
+      </c>
+      <c r="D121" s="5" t="inlineStr">
+        <is>
+          <t>Essential ECG Skills in the ER 1</t>
+        </is>
+      </c>
+      <c r="E121" s="4" t="inlineStr">
+        <is>
+          <t>579728</t>
+        </is>
+      </c>
+      <c r="F121" s="6" t="inlineStr">
+        <is>
+          <t>https://vimeo.com/1214919281</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="2" t="inlineStr">
+        <is>
+          <t>Kazuhito Hirata</t>
+        </is>
+      </c>
+      <c r="B122" s="2" t="inlineStr">
+        <is>
+          <t>循環器内科</t>
+        </is>
+      </c>
+      <c r="C122" s="3" t="inlineStr">
+        <is>
+          <t>社会福祉法人友愛会 友愛医療センター</t>
+        </is>
+      </c>
+      <c r="D122" s="3" t="inlineStr">
+        <is>
+          <t>Don't Miss Occult STEMI!</t>
+        </is>
+      </c>
+      <c r="E122" s="2" t="inlineStr">
+        <is>
+          <t>353300</t>
+        </is>
+      </c>
+      <c r="F122" s="7" t="inlineStr">
+        <is>
+          <t>https://vimeo.com/1214919431</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="4" t="inlineStr">
+        <is>
+          <t>Kazuhito Hirata</t>
+        </is>
+      </c>
+      <c r="B123" s="4" t="inlineStr">
+        <is>
+          <t>循環器内科</t>
+        </is>
+      </c>
+      <c r="C123" s="5" t="inlineStr">
+        <is>
+          <t>社会福祉法人友愛会 友愛医療センター</t>
+        </is>
+      </c>
+      <c r="D123" s="5" t="inlineStr">
+        <is>
+          <t>Auscultation Workshop (Diastolic Murmurs and Friction Rub)</t>
+        </is>
+      </c>
+      <c r="E123" s="4" t="inlineStr">
+        <is>
+          <t>687971</t>
+        </is>
+      </c>
+      <c r="F123" s="6" t="inlineStr">
+        <is>
+          <t>https://vimeo.com/1214919536</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="2" t="inlineStr">
+        <is>
+          <t>Kazuhito Hirata</t>
+        </is>
+      </c>
+      <c r="B124" s="2" t="inlineStr">
+        <is>
+          <t>循環器内科</t>
+        </is>
+      </c>
+      <c r="C124" s="3" t="inlineStr">
+        <is>
+          <t>社会福祉法人友愛会 友愛医療センター</t>
+        </is>
+      </c>
+      <c r="D124" s="3" t="inlineStr">
+        <is>
+          <t>Essential ECG Skills in the ER 2</t>
+        </is>
+      </c>
+      <c r="E124" s="2" t="inlineStr">
+        <is>
+          <t>579728</t>
+        </is>
+      </c>
+      <c r="F124" s="7" t="inlineStr">
+        <is>
+          <t>https://vimeo.com/1214919645</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="4" t="inlineStr">
+        <is>
+          <t>Dr. Richard McCartin</t>
+        </is>
+      </c>
+      <c r="B125" s="4" t="inlineStr">
+        <is>
+          <t>産婦人科</t>
+        </is>
+      </c>
+      <c r="C125" s="5" t="inlineStr">
+        <is>
+          <t>Assistant Professor, Department of Obstetrics and Gynecology, John A. Burns School of Medicine, University of Hawaii</t>
+        </is>
+      </c>
+      <c r="D125" s="5" t="inlineStr">
+        <is>
+          <t>Understanding the characteristics of energy devices and their safe use in surgery</t>
+        </is>
+      </c>
+      <c r="E125" s="4" t="inlineStr">
+        <is>
+          <t>154785</t>
+        </is>
+      </c>
+      <c r="F125" s="6" t="inlineStr">
+        <is>
+          <t>https://vimeo.com/1220355023</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="2" t="inlineStr">
+        <is>
+          <t>Dr. Richard McCartin</t>
+        </is>
+      </c>
+      <c r="B126" s="2" t="inlineStr">
+        <is>
+          <t>産婦人科</t>
+        </is>
+      </c>
+      <c r="C126" s="3" t="inlineStr">
+        <is>
+          <t>Assistant Professor, Department of Obstetrics and Gynecology, John A. Burns School of Medicine, University of Hawaii</t>
+        </is>
+      </c>
+      <c r="D126" s="3" t="inlineStr">
+        <is>
+          <t>Management of uterine fibroids and endometriosis</t>
+        </is>
+      </c>
+      <c r="E126" s="2" t="inlineStr">
+        <is>
+          <t>154785</t>
+        </is>
+      </c>
+      <c r="F126" s="7" t="inlineStr">
+        <is>
+          <t>https://vimeo.com/1220355173</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="4" t="inlineStr">
+        <is>
+          <t>Dr. Richard McCartin</t>
+        </is>
+      </c>
+      <c r="B127" s="4" t="inlineStr">
+        <is>
+          <t>産婦人科</t>
+        </is>
+      </c>
+      <c r="C127" s="5" t="inlineStr">
+        <is>
+          <t>Assistant Professor, Department of Obstetrics and Gynecology, John A. Burns School of Medicine, University of Hawaii</t>
+        </is>
+      </c>
+      <c r="D127" s="5" t="inlineStr">
+        <is>
+          <t>Patient safety</t>
+        </is>
+      </c>
+      <c r="E127" s="4" t="inlineStr">
+        <is>
+          <t>154785</t>
+        </is>
+      </c>
+      <c r="F127" s="6" t="inlineStr">
+        <is>
+          <t>https://vimeo.com/1220355314</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="2" t="inlineStr">
+        <is>
+          <t>Dr. Richard McCartin</t>
+        </is>
+      </c>
+      <c r="B128" s="2" t="inlineStr">
+        <is>
+          <t>産婦人科</t>
+        </is>
+      </c>
+      <c r="C128" s="3" t="inlineStr">
+        <is>
+          <t>Assistant Professor, Department of Obstetrics and Gynecology, John A. Burns School of Medicine, University of Hawaii</t>
+        </is>
+      </c>
+      <c r="D128" s="3" t="inlineStr">
+        <is>
+          <t>Management of ovarian cysts</t>
+        </is>
+      </c>
+      <c r="E128" s="2" t="inlineStr">
+        <is>
+          <t>154785</t>
+        </is>
+      </c>
+      <c r="F128" s="7" t="inlineStr">
+        <is>
+          <t>https://vimeo.com/1220355441</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="4" t="inlineStr">
+        <is>
+          <t>Dr. Richard McCartin</t>
+        </is>
+      </c>
+      <c r="B129" s="4" t="inlineStr">
+        <is>
+          <t>産婦人科</t>
+        </is>
+      </c>
+      <c r="C129" s="5" t="inlineStr">
+        <is>
+          <t>Assistant Professor, Department of Obstetrics and Gynecology, John A. Burns School of Medicine, University of Hawaii</t>
+        </is>
+      </c>
+      <c r="D129" s="5" t="inlineStr">
+        <is>
+          <t>Enhanced Recovery After Surgery (ERAS)</t>
+        </is>
+      </c>
+      <c r="E129" s="4" t="inlineStr">
+        <is>
+          <t>154785</t>
+        </is>
+      </c>
+      <c r="F129" s="6" t="inlineStr">
+        <is>
+          <t>https://vimeo.com/1220355502</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="2" t="inlineStr">
+        <is>
+          <t>Dr. Richard McCartin</t>
+        </is>
+      </c>
+      <c r="B130" s="2" t="inlineStr">
+        <is>
+          <t>産婦人科</t>
+        </is>
+      </c>
+      <c r="C130" s="3" t="inlineStr">
+        <is>
+          <t>Assistant Professor, Department of Obstetrics and Gynecology, John A. Burns School of Medicine, University of Hawaii</t>
+        </is>
+      </c>
+      <c r="D130" s="3" t="inlineStr">
+        <is>
+          <t>Case Conference: A Case of Tubo-Ovarian Abscess (TOA) Successfully Treated with Antibiotics Following Prolonged Mirena IUD Placement</t>
+        </is>
+      </c>
+      <c r="E130" s="2" t="inlineStr">
+        <is>
+          <t>426411</t>
+        </is>
+      </c>
+      <c r="F130" s="2" t="inlineStr"/>
+    </row>
+    <row r="131">
+      <c r="A131" s="4" t="inlineStr">
+        <is>
+          <t>Dr. Richard McCartin</t>
+        </is>
+      </c>
+      <c r="B131" s="4" t="inlineStr">
+        <is>
+          <t>産婦人科</t>
+        </is>
+      </c>
+      <c r="C131" s="5" t="inlineStr">
+        <is>
+          <t>Assistant Professor, Department of Obstetrics and Gynecology, John A. Burns School of Medicine, University of Hawaii</t>
+        </is>
+      </c>
+      <c r="D131" s="5" t="inlineStr">
+        <is>
+          <t>Case Conference: A Case of Tubo-Ovarian Abscess (TOA) with Difficult Antibiotic Selection Due to Drug Allergy</t>
+        </is>
+      </c>
+      <c r="E131" s="4" t="inlineStr">
+        <is>
+          <t>426411</t>
+        </is>
+      </c>
+      <c r="F131" s="4" t="inlineStr"/>
+    </row>
+    <row r="132">
+      <c r="A132" s="2" t="inlineStr">
+        <is>
+          <t>Dr. Joel Branch</t>
+        </is>
+      </c>
+      <c r="B132" s="2" t="inlineStr">
+        <is>
+          <t>内科</t>
+        </is>
+      </c>
+      <c r="C132" s="3" t="inlineStr">
+        <is>
+          <t>Director, Internal Medicine. Education &amp; Simulation Skills Training. Shonan Kamakura General Hosp. Director of Clinical Education Yao Tokushukai General Hospital</t>
+        </is>
+      </c>
+      <c r="D132" s="3" t="inlineStr">
+        <is>
+          <t>Sudden headache in α 52-yaer-old Female with migraine</t>
+        </is>
+      </c>
+      <c r="E132" s="2" t="inlineStr">
+        <is>
+          <t>587530</t>
+        </is>
+      </c>
+      <c r="F132" s="7" t="inlineStr">
+        <is>
+          <t>https://vimeo.com/1224759008</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="4" t="inlineStr">
+        <is>
+          <t>Dr. Joel Branch</t>
+        </is>
+      </c>
+      <c r="B133" s="4" t="inlineStr">
+        <is>
+          <t>内科</t>
+        </is>
+      </c>
+      <c r="C133" s="5" t="inlineStr">
+        <is>
+          <t>Director, Internal Medicine. Education &amp; Simulation Skills Training. Shonan Kamakura General Hosp. Director of Clinical Education Yao Tokushukai General Hospital</t>
+        </is>
+      </c>
+      <c r="D133" s="5" t="inlineStr">
+        <is>
+          <t>61-year-old male, impaired consciousness</t>
+        </is>
+      </c>
+      <c r="E133" s="4" t="inlineStr">
+        <is>
+          <t>587530</t>
+        </is>
+      </c>
+      <c r="F133" s="6" t="inlineStr">
+        <is>
+          <t>https://vimeo.com/1224759201</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="2" t="inlineStr">
+        <is>
+          <t>Dr. Joel Branch</t>
+        </is>
+      </c>
+      <c r="B134" s="2" t="inlineStr">
+        <is>
+          <t>内科</t>
+        </is>
+      </c>
+      <c r="C134" s="3" t="inlineStr">
+        <is>
+          <t>Director, Internal Medicine. Education &amp; Simulation Skills Training. Shonan Kamakura General Hosp. Director of Clinical Education Yao Tokushukai General Hospital</t>
+        </is>
+      </c>
+      <c r="D134" s="3" t="inlineStr">
+        <is>
+          <t>Important nail signs</t>
+        </is>
+      </c>
+      <c r="E134" s="2" t="inlineStr">
+        <is>
+          <t>300032</t>
+        </is>
+      </c>
+      <c r="F134" s="7" t="inlineStr">
+        <is>
+          <t>https://vimeo.com/1224759433</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="4" t="inlineStr">
+        <is>
+          <t>Dr. Joel Branch</t>
+        </is>
+      </c>
+      <c r="B135" s="4" t="inlineStr">
+        <is>
+          <t>内科</t>
+        </is>
+      </c>
+      <c r="C135" s="5" t="inlineStr">
+        <is>
+          <t>Director, Internal Medicine. Education &amp; Simulation Skills Training. Shonan Kamakura General Hosp. Director of Clinical Education Yao Tokushukai General Hospital</t>
+        </is>
+      </c>
+      <c r="D135" s="5" t="inlineStr">
+        <is>
+          <t>32-year-old Female with Headache</t>
+        </is>
+      </c>
+      <c r="E135" s="4" t="inlineStr">
+        <is>
+          <t>587530</t>
+        </is>
+      </c>
+      <c r="F135" s="6" t="inlineStr">
+        <is>
+          <t>https://vimeo.com/1224759676</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="2" t="inlineStr">
+        <is>
+          <t>Dr. Joel Branch</t>
+        </is>
+      </c>
+      <c r="B136" s="2" t="inlineStr">
+        <is>
+          <t>内科</t>
+        </is>
+      </c>
+      <c r="C136" s="3" t="inlineStr">
+        <is>
+          <t>Director, Internal Medicine. Education &amp; Simulation Skills Training. Shonan Kamakura General Hosp. Director of Clinical Education Yao Tokushukai General Hospital</t>
+        </is>
+      </c>
+      <c r="D136" s="3" t="inlineStr">
+        <is>
+          <t>Why the stethoscope is still an intrinsic tool of a physician</t>
+        </is>
+      </c>
+      <c r="E136" s="2" t="inlineStr">
+        <is>
+          <t>300032</t>
+        </is>
+      </c>
+      <c r="F136" s="7" t="inlineStr">
+        <is>
+          <t>https://vimeo.com/1224759857</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="4" t="inlineStr">
+        <is>
+          <t>Dr. Joel Branch</t>
+        </is>
+      </c>
+      <c r="B137" s="4" t="inlineStr">
+        <is>
+          <t>内科</t>
+        </is>
+      </c>
+      <c r="C137" s="5" t="inlineStr">
+        <is>
+          <t>Director, Internal Medicine. Education &amp; Simulation Skills Training. Shonan Kamakura General Hosp. Director of Clinical Education Yao Tokushukai General Hospital</t>
+        </is>
+      </c>
+      <c r="D137" s="5" t="inlineStr">
+        <is>
+          <t>74-year-old woman with altered behavior and progressive gait disturbance</t>
+        </is>
+      </c>
+      <c r="E137" s="4" t="inlineStr">
+        <is>
+          <t>587530</t>
+        </is>
+      </c>
+      <c r="F137" s="6" t="inlineStr">
+        <is>
+          <t>https://vimeo.com/1224760011</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="2" t="inlineStr">
+        <is>
+          <t>Dr. Joel Branch</t>
+        </is>
+      </c>
+      <c r="B138" s="2" t="inlineStr">
+        <is>
+          <t>内科</t>
+        </is>
+      </c>
+      <c r="C138" s="3" t="inlineStr">
+        <is>
+          <t>Director, Internal Medicine. Education &amp; Simulation Skills Training. Shonan Kamakura General Hosp. Director of Clinical Education Yao Tokushukai General Hospital</t>
+        </is>
+      </c>
+      <c r="D138" s="3" t="inlineStr">
+        <is>
+          <t>Treatment Paralysis</t>
+        </is>
+      </c>
+      <c r="E138" s="2" t="inlineStr">
+        <is>
+          <t>300032</t>
+        </is>
+      </c>
+      <c r="F138" s="7" t="inlineStr">
+        <is>
+          <t>https://vimeo.com/1224760583</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="4" t="inlineStr">
+        <is>
+          <t>Dr. Joel Branch</t>
+        </is>
+      </c>
+      <c r="B139" s="4" t="inlineStr">
+        <is>
+          <t>内科</t>
+        </is>
+      </c>
+      <c r="C139" s="5" t="inlineStr">
+        <is>
+          <t>Director, Internal Medicine. Education &amp; Simulation Skills Training. Shonan Kamakura General Hosp. Director of Clinical Education Yao Tokushukai General Hospital</t>
+        </is>
+      </c>
+      <c r="D139" s="5" t="inlineStr">
+        <is>
+          <t>74-year-old man, dyspnea with chest pain</t>
+        </is>
+      </c>
+      <c r="E139" s="4" t="inlineStr">
+        <is>
+          <t>587530</t>
+        </is>
+      </c>
+      <c r="F139" s="6" t="inlineStr">
+        <is>
+          <t>https://vimeo.com/1224760864</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="8" t="inlineStr">
+        <is>
+          <t>Dr.Amteshwar Singh</t>
+        </is>
+      </c>
+      <c r="B140" s="8" t="inlineStr">
+        <is>
+          <t>内科コンサルタント</t>
+        </is>
+      </c>
+      <c r="C140" s="3" t="inlineStr">
+        <is>
+          <t>Assistant Professor of Medicine, Johns Hopkins University School of Medicine / Director of Education, Division of Hospital Medicine</t>
+        </is>
+      </c>
+      <c r="D140" s="3" t="inlineStr">
+        <is>
+          <t>Physical Examination-The Why, The How, and The New Tools</t>
+        </is>
+      </c>
+      <c r="E140" s="8" t="inlineStr">
+        <is>
+          <t>245387</t>
+        </is>
+      </c>
+      <c r="F140" s="9" t="inlineStr">
+        <is>
+          <t>https://vimeo.com/1235238237</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="10" t="inlineStr">
+        <is>
+          <t>Dr.Amteshwar Singh</t>
+        </is>
+      </c>
+      <c r="B141" s="10" t="inlineStr">
+        <is>
+          <t>内科コンサルタント</t>
+        </is>
+      </c>
+      <c r="C141" s="5" t="inlineStr">
+        <is>
+          <t>Assistant Professor of Medicine, Johns Hopkins University School of Medicine / Director of Education, Division of Hospital Medicine</t>
+        </is>
+      </c>
+      <c r="D141" s="5" t="inlineStr">
+        <is>
+          <t>Neurologic Examination in a patient with left sided weakness</t>
+        </is>
+      </c>
+      <c r="E141" s="10" t="inlineStr">
+        <is>
+          <t>313180</t>
+        </is>
+      </c>
+      <c r="F141" s="11" t="inlineStr">
+        <is>
+          <t>https://vimeo.com/1235238485</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="8" t="inlineStr">
+        <is>
+          <t>Dr.Amteshwar Singh</t>
+        </is>
+      </c>
+      <c r="B142" s="8" t="inlineStr">
+        <is>
+          <t>内科コンサルタント</t>
+        </is>
+      </c>
+      <c r="C142" s="3" t="inlineStr">
+        <is>
+          <t>Assistant Professor of Medicine, Johns Hopkins University School of Medicine / Director of Education, Division of Hospital Medicine</t>
+        </is>
+      </c>
+      <c r="D142" s="3" t="inlineStr">
+        <is>
+          <t>Isolated Nystagmus and Ataxia – Neurologic</t>
+        </is>
+      </c>
+      <c r="E142" s="8" t="inlineStr">
+        <is>
+          <t>245387</t>
+        </is>
+      </c>
+      <c r="F142" s="9" t="inlineStr">
+        <is>
+          <t>https://vimeo.com/1235238729</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="10" t="inlineStr">
+        <is>
+          <t>Dr.Amteshwar Singh</t>
+        </is>
+      </c>
+      <c r="B143" s="10" t="inlineStr">
+        <is>
+          <t>内科コンサルタント</t>
+        </is>
+      </c>
+      <c r="C143" s="5" t="inlineStr">
+        <is>
+          <t>Assistant Professor of Medicine, Johns Hopkins University School of Medicine / Director of Education, Division of Hospital Medicine</t>
+        </is>
+      </c>
+      <c r="D143" s="5" t="inlineStr">
+        <is>
+          <t>Painful Weakness and Edema of the Legs – Neuromuscular Examination</t>
+        </is>
+      </c>
+      <c r="E143" s="10" t="inlineStr">
+        <is>
+          <t>245387</t>
+        </is>
+      </c>
+      <c r="F143" s="11" t="inlineStr">
+        <is>
+          <t>https://vimeo.com/1235239059</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="8" t="inlineStr">
+        <is>
+          <t>Dr.Amteshwar Singh</t>
+        </is>
+      </c>
+      <c r="B144" s="8" t="inlineStr">
+        <is>
+          <t>内科コンサルタント</t>
+        </is>
+      </c>
+      <c r="C144" s="3" t="inlineStr">
+        <is>
+          <t>Assistant Professor of Medicine, Johns Hopkins University School of Medicine / Director of Education, Division of Hospital Medicine</t>
+        </is>
+      </c>
+      <c r="D144" s="3" t="inlineStr">
+        <is>
+          <t>Examining joints in a patient with acute monoarticular swelling</t>
+        </is>
+      </c>
+      <c r="E144" s="8" t="inlineStr">
+        <is>
+          <t>313180</t>
+        </is>
+      </c>
+      <c r="F144" s="9" t="inlineStr">
+        <is>
+          <t>https://vimeo.com/1235239404</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="10" t="inlineStr">
+        <is>
+          <t>Dr.Amteshwar Singh</t>
+        </is>
+      </c>
+      <c r="B145" s="10" t="inlineStr">
+        <is>
+          <t>内科コンサルタント</t>
+        </is>
+      </c>
+      <c r="C145" s="5" t="inlineStr">
+        <is>
+          <t>Assistant Professor of Medicine, Johns Hopkins University School of Medicine / Director of Education, Division of Hospital Medicine</t>
+        </is>
+      </c>
+      <c r="D145" s="5" t="inlineStr">
+        <is>
+          <t>Adult-Onset Chorea in a geriatric patient – Neurologic</t>
+        </is>
+      </c>
+      <c r="E145" s="10" t="inlineStr">
+        <is>
+          <t>245387</t>
+        </is>
+      </c>
+      <c r="F145" s="11" t="inlineStr">
+        <is>
+          <t>https://vimeo.com/1235239662</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="8" t="inlineStr">
+        <is>
+          <t>Dr.Amteshwar Singh</t>
+        </is>
+      </c>
+      <c r="B146" s="8" t="inlineStr">
+        <is>
+          <t>内科コンサルタント</t>
+        </is>
+      </c>
+      <c r="C146" s="3" t="inlineStr">
+        <is>
+          <t>Assistant Professor of Medicine, Johns Hopkins University School of Medicine / Director of Education, Division of Hospital Medicine</t>
+        </is>
+      </c>
+      <c r="D146" s="3" t="inlineStr">
+        <is>
+          <t>Examining the heart in a patient with dyspnea on exertion and pedal edema</t>
+        </is>
+      </c>
+      <c r="E146" s="8" t="inlineStr">
+        <is>
+          <t>313180</t>
+        </is>
+      </c>
+      <c r="F146" s="9" t="inlineStr">
+        <is>
+          <t>https://vimeo.com/1235239924</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="10" t="inlineStr">
+        <is>
+          <t>Dr.Amteshwar Singh</t>
+        </is>
+      </c>
+      <c r="B147" s="10" t="inlineStr">
+        <is>
+          <t>内科コンサルタント</t>
+        </is>
+      </c>
+      <c r="C147" s="5" t="inlineStr">
+        <is>
+          <t>Assistant Professor of Medicine, Johns Hopkins University School of Medicine / Director of Education, Division of Hospital Medicine</t>
+        </is>
+      </c>
+      <c r="D147" s="5" t="inlineStr">
+        <is>
+          <t>Unresolving pneumonia needing a diagnostic time out</t>
+        </is>
+      </c>
+      <c r="E147" s="10" t="inlineStr">
+        <is>
+          <t>245387</t>
+        </is>
+      </c>
+      <c r="F147" s="11" t="inlineStr">
+        <is>
+          <t>https://vimeo.com/1235240131</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="8" t="inlineStr">
+        <is>
+          <t>Dr.Amteshwar Singh</t>
+        </is>
+      </c>
+      <c r="B148" s="8" t="inlineStr">
+        <is>
+          <t>内科コンサルタント</t>
+        </is>
+      </c>
+      <c r="C148" s="3" t="inlineStr">
+        <is>
+          <t>Assistant Professor of Medicine, Johns Hopkins University School of Medicine / Director of Education, Division of Hospital Medicine</t>
+        </is>
+      </c>
+      <c r="D148" s="3" t="inlineStr">
+        <is>
+          <t>Respiratory Examination in a Dyspneic patient</t>
+        </is>
+      </c>
+      <c r="E148" s="8" t="inlineStr">
+        <is>
+          <t>313180</t>
+        </is>
+      </c>
+      <c r="F148" s="9" t="inlineStr">
+        <is>
+          <t>https://vimeo.com/1235240362</t>
         </is>
       </c>
     </row>
@@ -4024,6 +5077,36 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F112" r:id="rId73"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F113" r:id="rId74"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F115" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F116" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F117" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F119" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F120" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F121" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F122" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F123" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F124" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F125" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F126" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F127" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F128" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F129" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F132" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F133" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F134" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F135" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F136" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F137" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F138" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F139" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F140" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F141" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F142" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F143" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F144" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F145" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F146" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F147" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F148" r:id="rId105"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add Dr. Masanori Tei lecture and refresh gallery metadata
- Add Dr. Masanori Tei's (Saku Central Hospital) Oct 20-22 sessions and
  Dr. Satoshi Miyashita's Oct 28-30 sessions to consultant_vimeo.csv.
- Download Tei's 3 Zoom recordings, upload to Vimeo with passwords, and
  update vimeo_results.csv / vimeo_links.xlsx / vimeo_links_omit.xlsx.
- Regenerate vimeo_metadata_export.csv, which had not been refreshed since
  June: adds 33 videos (Hirata, McCartin, Branch, Singh, Tei) to the gallery
  and fixes Dr. Kana Miyata's affiliation.
- export_vimeo_metadata_csv.py: resolve Vimeo's relative paging.next URL;
  the export crashed once the account passed 100 videos.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/vimeo_links.xlsx
+++ b/vimeo_links.xlsx
@@ -64,7 +64,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -85,18 +85,6 @@
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
   </cellXfs>
@@ -464,7 +452,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F148"/>
+  <dimension ref="A1:F157"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -563,7 +551,7 @@
       </c>
       <c r="F3" s="6" t="inlineStr">
         <is>
-          <t>https://vimeo.com/1154200765</t>
+          <t>https://vimeo.com/1154202805</t>
         </is>
       </c>
     </row>
@@ -595,7 +583,7 @@
       </c>
       <c r="F4" s="7" t="inlineStr">
         <is>
-          <t>https://vimeo.com/1154200948</t>
+          <t>https://vimeo.com/1154202922</t>
         </is>
       </c>
     </row>
@@ -659,7 +647,7 @@
       </c>
       <c r="F6" s="7" t="inlineStr">
         <is>
-          <t>https://vimeo.com/1154203167</t>
+          <t>https://vimeo.com/1154203273</t>
         </is>
       </c>
     </row>
@@ -687,7 +675,7 @@
       <c r="E7" s="4" t="inlineStr"/>
       <c r="F7" s="6" t="inlineStr">
         <is>
-          <t>https://vimeo.com/1154203167</t>
+          <t>https://vimeo.com/1154203273</t>
         </is>
       </c>
     </row>
@@ -2871,7 +2859,7 @@
       </c>
       <c r="F80" s="7" t="inlineStr">
         <is>
-          <t>https://vimeo.com/1177162061</t>
+          <t>https://vimeo.com/1192449734</t>
         </is>
       </c>
     </row>
@@ -2903,7 +2891,7 @@
       </c>
       <c r="F81" s="6" t="inlineStr">
         <is>
-          <t>https://vimeo.com/1177162237</t>
+          <t>https://vimeo.com/1192449909</t>
         </is>
       </c>
     </row>
@@ -2935,7 +2923,7 @@
       </c>
       <c r="F82" s="7" t="inlineStr">
         <is>
-          <t>https://vimeo.com/1177162517</t>
+          <t>https://vimeo.com/1192450070</t>
         </is>
       </c>
     </row>
@@ -2967,7 +2955,7 @@
       </c>
       <c r="F83" s="6" t="inlineStr">
         <is>
-          <t>https://vimeo.com/1177162727</t>
+          <t>https://vimeo.com/1192450190</t>
         </is>
       </c>
     </row>
@@ -3643,7 +3631,7 @@
       </c>
       <c r="F105" s="6" t="inlineStr">
         <is>
-          <t>https://vimeo.com/1204027316</t>
+          <t>https://vimeo.com/1200665260</t>
         </is>
       </c>
     </row>
@@ -3940,7 +3928,7 @@
       </c>
       <c r="C115" s="5" t="inlineStr">
         <is>
-          <t>Associate Professor  Department of Internal Medicine
+          <t>Associate Professor  Department of Internal Medicine
          Division of Nephrology, St Louis University School of Medicine</t>
         </is>
       </c>
@@ -4713,12 +4701,12 @@
       </c>
     </row>
     <row r="140">
-      <c r="A140" s="8" t="inlineStr">
+      <c r="A140" s="2" t="inlineStr">
         <is>
           <t>Dr.Amteshwar Singh</t>
         </is>
       </c>
-      <c r="B140" s="8" t="inlineStr">
+      <c r="B140" s="2" t="inlineStr">
         <is>
           <t>内科コンサルタント</t>
         </is>
@@ -4733,24 +4721,24 @@
           <t>Physical Examination-The Why, The How, and The New Tools</t>
         </is>
       </c>
-      <c r="E140" s="8" t="inlineStr">
+      <c r="E140" s="2" t="inlineStr">
         <is>
           <t>245387</t>
         </is>
       </c>
-      <c r="F140" s="9" t="inlineStr">
+      <c r="F140" s="7" t="inlineStr">
         <is>
           <t>https://vimeo.com/1235238237</t>
         </is>
       </c>
     </row>
     <row r="141">
-      <c r="A141" s="10" t="inlineStr">
+      <c r="A141" s="4" t="inlineStr">
         <is>
           <t>Dr.Amteshwar Singh</t>
         </is>
       </c>
-      <c r="B141" s="10" t="inlineStr">
+      <c r="B141" s="4" t="inlineStr">
         <is>
           <t>内科コンサルタント</t>
         </is>
@@ -4765,24 +4753,24 @@
           <t>Neurologic Examination in a patient with left sided weakness</t>
         </is>
       </c>
-      <c r="E141" s="10" t="inlineStr">
+      <c r="E141" s="4" t="inlineStr">
         <is>
           <t>313180</t>
         </is>
       </c>
-      <c r="F141" s="11" t="inlineStr">
+      <c r="F141" s="6" t="inlineStr">
         <is>
           <t>https://vimeo.com/1235238485</t>
         </is>
       </c>
     </row>
     <row r="142">
-      <c r="A142" s="8" t="inlineStr">
+      <c r="A142" s="2" t="inlineStr">
         <is>
           <t>Dr.Amteshwar Singh</t>
         </is>
       </c>
-      <c r="B142" s="8" t="inlineStr">
+      <c r="B142" s="2" t="inlineStr">
         <is>
           <t>内科コンサルタント</t>
         </is>
@@ -4797,24 +4785,24 @@
           <t>Isolated Nystagmus and Ataxia – Neurologic</t>
         </is>
       </c>
-      <c r="E142" s="8" t="inlineStr">
+      <c r="E142" s="2" t="inlineStr">
         <is>
           <t>245387</t>
         </is>
       </c>
-      <c r="F142" s="9" t="inlineStr">
+      <c r="F142" s="7" t="inlineStr">
         <is>
           <t>https://vimeo.com/1235238729</t>
         </is>
       </c>
     </row>
     <row r="143">
-      <c r="A143" s="10" t="inlineStr">
+      <c r="A143" s="4" t="inlineStr">
         <is>
           <t>Dr.Amteshwar Singh</t>
         </is>
       </c>
-      <c r="B143" s="10" t="inlineStr">
+      <c r="B143" s="4" t="inlineStr">
         <is>
           <t>内科コンサルタント</t>
         </is>
@@ -4826,179 +4814,443 @@
       </c>
       <c r="D143" s="5" t="inlineStr">
         <is>
+          <t>The Importance of History-Taking and Physical Examination in the AI Era</t>
+        </is>
+      </c>
+      <c r="E143" s="4" t="inlineStr">
+        <is>
+          <t>307235</t>
+        </is>
+      </c>
+      <c r="F143" s="4" t="inlineStr"/>
+    </row>
+    <row r="144">
+      <c r="A144" s="2" t="inlineStr">
+        <is>
+          <t>Dr.Amteshwar Singh</t>
+        </is>
+      </c>
+      <c r="B144" s="2" t="inlineStr">
+        <is>
+          <t>内科コンサルタント</t>
+        </is>
+      </c>
+      <c r="C144" s="3" t="inlineStr">
+        <is>
+          <t>Assistant Professor of Medicine, Johns Hopkins University School of Medicine / Director of Education, Division of Hospital Medicine</t>
+        </is>
+      </c>
+      <c r="D144" s="3" t="inlineStr">
+        <is>
+          <t>Bedside Physical Examination-Centered Teaching Session</t>
+        </is>
+      </c>
+      <c r="E144" s="2" t="inlineStr">
+        <is>
+          <t>307235</t>
+        </is>
+      </c>
+      <c r="F144" s="2" t="inlineStr"/>
+    </row>
+    <row r="145">
+      <c r="A145" s="4" t="inlineStr">
+        <is>
+          <t>Dr.Amteshwar Singh</t>
+        </is>
+      </c>
+      <c r="B145" s="4" t="inlineStr">
+        <is>
+          <t>内科コンサルタント</t>
+        </is>
+      </c>
+      <c r="C145" s="5" t="inlineStr">
+        <is>
+          <t>Assistant Professor of Medicine, Johns Hopkins University School of Medicine / Director of Education, Division of Hospital Medicine</t>
+        </is>
+      </c>
+      <c r="D145" s="5" t="inlineStr">
+        <is>
           <t>Painful Weakness and Edema of the Legs – Neuromuscular Examination</t>
         </is>
       </c>
-      <c r="E143" s="10" t="inlineStr">
+      <c r="E145" s="4" t="inlineStr">
         <is>
           <t>245387</t>
         </is>
       </c>
-      <c r="F143" s="11" t="inlineStr">
+      <c r="F145" s="6" t="inlineStr">
         <is>
           <t>https://vimeo.com/1235239059</t>
         </is>
       </c>
     </row>
-    <row r="144">
-      <c r="A144" s="8" t="inlineStr">
+    <row r="146">
+      <c r="A146" s="2" t="inlineStr">
         <is>
           <t>Dr.Amteshwar Singh</t>
         </is>
       </c>
-      <c r="B144" s="8" t="inlineStr">
+      <c r="B146" s="2" t="inlineStr">
         <is>
           <t>内科コンサルタント</t>
         </is>
       </c>
-      <c r="C144" s="3" t="inlineStr">
+      <c r="C146" s="3" t="inlineStr">
         <is>
           <t>Assistant Professor of Medicine, Johns Hopkins University School of Medicine / Director of Education, Division of Hospital Medicine</t>
         </is>
       </c>
-      <c r="D144" s="3" t="inlineStr">
+      <c r="D146" s="3" t="inlineStr">
         <is>
           <t>Examining joints in a patient with acute monoarticular swelling</t>
         </is>
       </c>
-      <c r="E144" s="8" t="inlineStr">
+      <c r="E146" s="2" t="inlineStr">
         <is>
           <t>313180</t>
         </is>
       </c>
-      <c r="F144" s="9" t="inlineStr">
+      <c r="F146" s="7" t="inlineStr">
         <is>
           <t>https://vimeo.com/1235239404</t>
         </is>
       </c>
     </row>
-    <row r="145">
-      <c r="A145" s="10" t="inlineStr">
+    <row r="147">
+      <c r="A147" s="4" t="inlineStr">
         <is>
           <t>Dr.Amteshwar Singh</t>
         </is>
       </c>
-      <c r="B145" s="10" t="inlineStr">
+      <c r="B147" s="4" t="inlineStr">
         <is>
           <t>内科コンサルタント</t>
         </is>
       </c>
-      <c r="C145" s="5" t="inlineStr">
+      <c r="C147" s="5" t="inlineStr">
         <is>
           <t>Assistant Professor of Medicine, Johns Hopkins University School of Medicine / Director of Education, Division of Hospital Medicine</t>
         </is>
       </c>
-      <c r="D145" s="5" t="inlineStr">
+      <c r="D147" s="5" t="inlineStr">
         <is>
           <t>Adult-Onset Chorea in a geriatric patient – Neurologic</t>
         </is>
       </c>
-      <c r="E145" s="10" t="inlineStr">
+      <c r="E147" s="4" t="inlineStr">
         <is>
           <t>245387</t>
         </is>
       </c>
-      <c r="F145" s="11" t="inlineStr">
+      <c r="F147" s="6" t="inlineStr">
         <is>
           <t>https://vimeo.com/1235239662</t>
         </is>
       </c>
     </row>
-    <row r="146">
-      <c r="A146" s="8" t="inlineStr">
+    <row r="148">
+      <c r="A148" s="2" t="inlineStr">
         <is>
           <t>Dr.Amteshwar Singh</t>
         </is>
       </c>
-      <c r="B146" s="8" t="inlineStr">
+      <c r="B148" s="2" t="inlineStr">
         <is>
           <t>内科コンサルタント</t>
         </is>
       </c>
-      <c r="C146" s="3" t="inlineStr">
+      <c r="C148" s="3" t="inlineStr">
         <is>
           <t>Assistant Professor of Medicine, Johns Hopkins University School of Medicine / Director of Education, Division of Hospital Medicine</t>
         </is>
       </c>
-      <c r="D146" s="3" t="inlineStr">
+      <c r="D148" s="3" t="inlineStr">
         <is>
           <t>Examining the heart in a patient with dyspnea on exertion and pedal edema</t>
         </is>
       </c>
-      <c r="E146" s="8" t="inlineStr">
+      <c r="E148" s="2" t="inlineStr">
         <is>
           <t>313180</t>
         </is>
       </c>
-      <c r="F146" s="9" t="inlineStr">
+      <c r="F148" s="7" t="inlineStr">
         <is>
           <t>https://vimeo.com/1235239924</t>
         </is>
       </c>
     </row>
-    <row r="147">
-      <c r="A147" s="10" t="inlineStr">
+    <row r="149">
+      <c r="A149" s="4" t="inlineStr">
         <is>
           <t>Dr.Amteshwar Singh</t>
         </is>
       </c>
-      <c r="B147" s="10" t="inlineStr">
+      <c r="B149" s="4" t="inlineStr">
         <is>
           <t>内科コンサルタント</t>
         </is>
       </c>
-      <c r="C147" s="5" t="inlineStr">
+      <c r="C149" s="5" t="inlineStr">
         <is>
           <t>Assistant Professor of Medicine, Johns Hopkins University School of Medicine / Director of Education, Division of Hospital Medicine</t>
         </is>
       </c>
-      <c r="D147" s="5" t="inlineStr">
+      <c r="D149" s="5" t="inlineStr">
         <is>
           <t>Unresolving pneumonia needing a diagnostic time out</t>
         </is>
       </c>
-      <c r="E147" s="10" t="inlineStr">
+      <c r="E149" s="4" t="inlineStr">
         <is>
           <t>245387</t>
         </is>
       </c>
-      <c r="F147" s="11" t="inlineStr">
+      <c r="F149" s="6" t="inlineStr">
         <is>
           <t>https://vimeo.com/1235240131</t>
         </is>
       </c>
     </row>
-    <row r="148">
-      <c r="A148" s="8" t="inlineStr">
+    <row r="150">
+      <c r="A150" s="2" t="inlineStr">
         <is>
           <t>Dr.Amteshwar Singh</t>
         </is>
       </c>
-      <c r="B148" s="8" t="inlineStr">
+      <c r="B150" s="2" t="inlineStr">
         <is>
           <t>内科コンサルタント</t>
         </is>
       </c>
-      <c r="C148" s="3" t="inlineStr">
+      <c r="C150" s="3" t="inlineStr">
         <is>
           <t>Assistant Professor of Medicine, Johns Hopkins University School of Medicine / Director of Education, Division of Hospital Medicine</t>
         </is>
       </c>
-      <c r="D148" s="3" t="inlineStr">
+      <c r="D150" s="3" t="inlineStr">
         <is>
           <t>Respiratory Examination in a Dyspneic patient</t>
         </is>
       </c>
-      <c r="E148" s="8" t="inlineStr">
+      <c r="E150" s="2" t="inlineStr">
         <is>
           <t>313180</t>
         </is>
       </c>
-      <c r="F148" s="9" t="inlineStr">
+      <c r="F150" s="7" t="inlineStr">
         <is>
           <t>https://vimeo.com/1235240362</t>
         </is>
       </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="4" t="inlineStr">
+        <is>
+          <t>Dr. Masanori Tei</t>
+        </is>
+      </c>
+      <c r="B151" s="4" t="inlineStr">
+        <is>
+          <t>総合診療科</t>
+        </is>
+      </c>
+      <c r="C151" s="5" t="inlineStr">
+        <is>
+          <t>佐久総合病院 院長</t>
+        </is>
+      </c>
+      <c r="D151" s="5" t="inlineStr">
+        <is>
+          <t>Tips for Discharge Planning (Part 1): How to Proceed with Discharge Coordination</t>
+        </is>
+      </c>
+      <c r="E151" s="4" t="inlineStr">
+        <is>
+          <t>251480</t>
+        </is>
+      </c>
+      <c r="F151" s="6" t="inlineStr">
+        <is>
+          <t>https://vimeo.com/1238617595</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="2" t="inlineStr">
+        <is>
+          <t>Dr. Masanori Tei</t>
+        </is>
+      </c>
+      <c r="B152" s="2" t="inlineStr">
+        <is>
+          <t>総合診療科</t>
+        </is>
+      </c>
+      <c r="C152" s="3" t="inlineStr">
+        <is>
+          <t>佐久総合病院 院長</t>
+        </is>
+      </c>
+      <c r="D152" s="3" t="inlineStr">
+        <is>
+          <t>Role Sharing Among Hospitals in the Era of Community-Based Integrated Care</t>
+        </is>
+      </c>
+      <c r="E152" s="2" t="inlineStr">
+        <is>
+          <t>970652</t>
+        </is>
+      </c>
+      <c r="F152" s="7" t="inlineStr">
+        <is>
+          <t>https://vimeo.com/1238617738</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="4" t="inlineStr">
+        <is>
+          <t>Dr. Masanori Tei</t>
+        </is>
+      </c>
+      <c r="B153" s="4" t="inlineStr">
+        <is>
+          <t>総合診療科</t>
+        </is>
+      </c>
+      <c r="C153" s="5" t="inlineStr">
+        <is>
+          <t>佐久総合病院 院長</t>
+        </is>
+      </c>
+      <c r="D153" s="5" t="inlineStr">
+        <is>
+          <t>Tips for Discharge Planning (Part 2): Choosing the Place of Care After Acute Treatment</t>
+        </is>
+      </c>
+      <c r="E153" s="4" t="inlineStr">
+        <is>
+          <t>251480</t>
+        </is>
+      </c>
+      <c r="F153" s="6" t="inlineStr">
+        <is>
+          <t>https://vimeo.com/1238618109</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="2" t="inlineStr">
+        <is>
+          <t>Dr. Satoshi Miyashita</t>
+        </is>
+      </c>
+      <c r="B154" s="2" t="inlineStr">
+        <is>
+          <t>集中治療科</t>
+        </is>
+      </c>
+      <c r="C154" s="3" t="inlineStr">
+        <is>
+          <t>Assistant Professor, Department of Cardiovascular Medicine, Dartmouth Hitchcock Medical Center</t>
+        </is>
+      </c>
+      <c r="D154" s="3" t="inlineStr">
+        <is>
+          <t>Cardiac Critical Care and Heart Failure in the United States</t>
+        </is>
+      </c>
+      <c r="E154" s="2" t="inlineStr">
+        <is>
+          <t>511990</t>
+        </is>
+      </c>
+      <c r="F154" s="2" t="inlineStr"/>
+    </row>
+    <row r="155">
+      <c r="A155" s="4" t="inlineStr">
+        <is>
+          <t>Dr. Satoshi Miyashita</t>
+        </is>
+      </c>
+      <c r="B155" s="4" t="inlineStr">
+        <is>
+          <t>集中治療科</t>
+        </is>
+      </c>
+      <c r="C155" s="5" t="inlineStr">
+        <is>
+          <t>Assistant Professor, Department of Cardiovascular Medicine, Dartmouth Hitchcock Medical Center</t>
+        </is>
+      </c>
+      <c r="D155" s="5" t="inlineStr">
+        <is>
+          <t>Heart Failure Management: Questioning Conventional Wisdom</t>
+        </is>
+      </c>
+      <c r="E155" s="4" t="inlineStr">
+        <is>
+          <t>323011</t>
+        </is>
+      </c>
+      <c r="F155" s="4" t="inlineStr"/>
+    </row>
+    <row r="156">
+      <c r="A156" s="2" t="inlineStr">
+        <is>
+          <t>Dr. Satoshi Miyashita</t>
+        </is>
+      </c>
+      <c r="B156" s="2" t="inlineStr">
+        <is>
+          <t>集中治療科</t>
+        </is>
+      </c>
+      <c r="C156" s="3" t="inlineStr">
+        <is>
+          <t>Assistant Professor, Department of Cardiovascular Medicine, Dartmouth Hitchcock Medical Center</t>
+        </is>
+      </c>
+      <c r="D156" s="3" t="inlineStr">
+        <is>
+          <t>Cardiac Critical Care and Mechanical Ventilation Management</t>
+        </is>
+      </c>
+      <c r="E156" s="2" t="inlineStr">
+        <is>
+          <t>251480</t>
+        </is>
+      </c>
+      <c r="F156" s="2" t="inlineStr"/>
+    </row>
+    <row r="157">
+      <c r="A157" s="4" t="inlineStr">
+        <is>
+          <t>Dr. Satoshi Miyashita</t>
+        </is>
+      </c>
+      <c r="B157" s="4" t="inlineStr">
+        <is>
+          <t>集中治療科</t>
+        </is>
+      </c>
+      <c r="C157" s="5" t="inlineStr">
+        <is>
+          <t>Assistant Professor, Department of Cardiovascular Medicine, Dartmouth Hitchcock Medical Center</t>
+        </is>
+      </c>
+      <c r="D157" s="5" t="inlineStr">
+        <is>
+          <t>Impella Treatment Strategy with a Long-Term Perspective</t>
+        </is>
+      </c>
+      <c r="E157" s="4" t="inlineStr">
+        <is>
+          <t>323011</t>
+        </is>
+      </c>
+      <c r="F157" s="4" t="inlineStr"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -5101,12 +5353,15 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F140" r:id="rId97"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F141" r:id="rId98"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F142" r:id="rId99"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F143" r:id="rId100"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F144" r:id="rId101"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F145" r:id="rId102"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F146" r:id="rId103"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F147" r:id="rId104"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F148" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F145" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F146" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F147" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F148" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F149" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F150" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F151" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F152" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F153" r:id="rId108"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>